<commit_message>
Before changes Working Code
</commit_message>
<xml_diff>
--- a/src/test/resources/TestData.xlsx
+++ b/src/test/resources/TestData.xlsx
@@ -3,24 +3,25 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <mc:AlternateContent>
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SathishReddy Sandhi\SeleniumAutomation\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9942B1D7-3B81-4C87-944B-6DB53D4A4507}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D43A39F-BBF0-4140-B8BE-DA360D2B1864}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dashboard" sheetId="2" r:id="rId1"/>
     <sheet name="Cart" sheetId="3" r:id="rId2"/>
     <sheet name="Payment" sheetId="4" r:id="rId3"/>
     <sheet name="Order" sheetId="5" r:id="rId4"/>
+    <sheet name="Results" sheetId="6" r:id="rId5"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
   </extLst>
@@ -28,60 +29,73 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="20">
   <si>
     <t>ProductName</t>
   </si>
   <si>
-    <t>ProductCount</t>
-  </si>
-  <si>
-    <t>CerditCardNumber</t>
-  </si>
-  <si>
-    <t>exp Month</t>
-  </si>
-  <si>
-    <t>exp Date</t>
-  </si>
-  <si>
     <t>CVV</t>
   </si>
   <si>
-    <t>NameOnCard</t>
-  </si>
-  <si>
     <t>Country</t>
   </si>
   <si>
     <t>iphone 13 pro</t>
   </si>
   <si>
-    <t>1234567890987650</t>
-  </si>
-  <si>
-    <t>12</t>
-  </si>
-  <si>
-    <t>31</t>
-  </si>
-  <si>
-    <t>274</t>
-  </si>
-  <si>
     <t>Sathish Reddy</t>
   </si>
   <si>
     <t>India</t>
   </si>
   <si>
-    <t>1</t>
+    <t>ExpectedCartCount</t>
+  </si>
+  <si>
+    <t>CardNumber</t>
+  </si>
+  <si>
+    <t>Month</t>
+  </si>
+  <si>
+    <t>Date</t>
+  </si>
+  <si>
+    <t>Name</t>
+  </si>
+  <si>
+    <t>ExpectedQty</t>
+  </si>
+  <si>
+    <t>ZARA COAT 3</t>
+  </si>
+  <si>
+    <t>Sathish Reddy Sandhi</t>
+  </si>
+  <si>
+    <t>1234567898765432</t>
+  </si>
+  <si>
+    <t>09</t>
+  </si>
+  <si>
+    <t>E2ETest</t>
+  </si>
+  <si>
+    <t>CompletedFlow</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>Cart.goToCheckout</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="0"/>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -91,12 +105,32 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="none">
+        <fgColor indexed="17"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor indexed="17"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="none">
+        <fgColor indexed="10"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor indexed="10"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -111,9 +145,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="true"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -394,27 +433,35 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CF2D4A01-FD8A-4C00-8AEF-6100DA0E02DE}">
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B3"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="14.1796875" customWidth="1"/>
-    <col min="2" max="2" width="13.54296875" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="14.1796875"/>
+    <col min="2" max="2" customWidth="true" width="23.08984375"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
+      <c r="A1" t="s" s="0">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" t="s" s="0">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A2" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="B2" s="1">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>15</v>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A3" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="B3" s="1">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -424,23 +471,34 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{334CF848-C880-4642-954D-864DF5E51C2D}">
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B3"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="2" max="2" customWidth="true" width="19.90625"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
+      <c r="A1" t="s" s="0">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" t="s" s="0">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A2" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="B2" s="1">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>15</v>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A3" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="B3" s="1">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -451,53 +509,73 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B2AF52E-5086-43AC-9E41-3304A02A9C8C}">
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="36.26953125" customWidth="1"/>
-    <col min="2" max="2" width="12.6328125" customWidth="1"/>
-    <col min="5" max="5" width="23.1796875" customWidth="1"/>
-    <col min="6" max="6" width="13.1796875" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="23.81640625"/>
+    <col min="2" max="2" customWidth="true" width="12.6328125"/>
+    <col min="5" max="5" customWidth="true" width="23.1796875"/>
+    <col min="6" max="6" customWidth="true" width="13.1796875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
+      <c r="A1" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="B1" t="s" s="0">
+        <v>8</v>
+      </c>
+      <c r="C1" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D1" t="s" s="0">
+        <v>1</v>
+      </c>
+      <c r="E1" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="F1" t="s" s="0">
         <v>2</v>
-      </c>
-      <c r="B1" t="s">
-        <v>3</v>
-      </c>
-      <c r="C1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D1" t="s">
-        <v>5</v>
-      </c>
-      <c r="E1" t="s">
-        <v>6</v>
-      </c>
-      <c r="F1" t="s">
-        <v>7</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B2" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B2" s="1">
+        <v>12</v>
+      </c>
+      <c r="C2" s="1">
+        <v>31</v>
+      </c>
+      <c r="D2" s="1">
+        <v>274</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F2" t="s" s="0">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A3" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" s="1">
         <v>10</v>
       </c>
-      <c r="C2" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="E2" s="1" t="s">
+      <c r="D3" s="1">
+        <v>294</v>
+      </c>
+      <c r="E3" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="F2" t="s">
-        <v>14</v>
+      <c r="F3" t="s" s="0">
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -507,27 +585,89 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4E14915E-E896-4209-8E48-035EA63E22E1}">
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B3"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="16.1796875" customWidth="1"/>
-    <col min="2" max="2" width="16.7265625" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="16.1796875"/>
+    <col min="2" max="2" customWidth="true" width="36.90625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
+      <c r="A1" t="s" s="0">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" t="s" s="0">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A2" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="B2" s="1">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>15</v>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A3" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="B3" s="1">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F7FAC67C-2142-481E-8C57-BF49024F7BB1}">
+  <dimension ref="A1:C5"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="2">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="3">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="B3" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="C3" t="s" s="4">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="B4" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="C4" t="s" s="5">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="B5" t="s" s="0">
+        <v>19</v>
+      </c>
+      <c r="C5" t="s" s="6">
+        <v>18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
EndToEND Flow with all utilities
</commit_message>
<xml_diff>
--- a/src/test/resources/TestData.xlsx
+++ b/src/test/resources/TestData.xlsx
@@ -8,16 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SathishReddy Sandhi\SeleniumAutomation\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D43A39F-BBF0-4140-B8BE-DA360D2B1864}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05B21351-D445-4ACC-B24F-292D7CEB8FCF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Dashboard" sheetId="2" r:id="rId1"/>
-    <sheet name="Cart" sheetId="3" r:id="rId2"/>
-    <sheet name="Payment" sheetId="4" r:id="rId3"/>
-    <sheet name="Order" sheetId="5" r:id="rId4"/>
-    <sheet name="Results" sheetId="6" r:id="rId5"/>
+    <sheet name="Results" sheetId="8" r:id="rId1"/>
+    <sheet name="Dashboard" sheetId="2" r:id="rId2"/>
+    <sheet name="Cart" sheetId="3" r:id="rId3"/>
+    <sheet name="Payment" sheetId="4" r:id="rId4"/>
+    <sheet name="Order" sheetId="5" r:id="rId5"/>
+    <sheet name="shipmnent" sheetId="7" r:id="rId6"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -29,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="36">
   <si>
     <t>ProductName</t>
   </si>
@@ -40,62 +41,113 @@
     <t>Country</t>
   </si>
   <si>
+    <t>Sathish Reddy</t>
+  </si>
+  <si>
+    <t>India</t>
+  </si>
+  <si>
+    <t>ExpectedCartCount</t>
+  </si>
+  <si>
+    <t>CardNumber</t>
+  </si>
+  <si>
+    <t>Month</t>
+  </si>
+  <si>
+    <t>Date</t>
+  </si>
+  <si>
+    <t>Name</t>
+  </si>
+  <si>
+    <t>ExpectedQty</t>
+  </si>
+  <si>
+    <t>Sathish Reddy Sandhi</t>
+  </si>
+  <si>
+    <t>1234567898765432</t>
+  </si>
+  <si>
+    <t>09</t>
+  </si>
+  <si>
+    <t>Address</t>
+  </si>
+  <si>
+    <t>landmark</t>
+  </si>
+  <si>
+    <t>vlmp</t>
+  </si>
+  <si>
+    <t>hanuman temple</t>
+  </si>
+  <si>
+    <t>1234564898765437</t>
+  </si>
+  <si>
+    <t>06</t>
+  </si>
+  <si>
+    <t>Devender Reddy</t>
+  </si>
+  <si>
+    <t>E2ETest</t>
+  </si>
+  <si>
+    <t>FAIL</t>
+  </si>
+  <si>
+    <t>Cart.goToCheckout</t>
+  </si>
+  <si>
+    <t>ZARA COAT 3</t>
+  </si>
+  <si>
+    <t>TestCaseName</t>
+  </si>
+  <si>
+    <t>StepName</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>Timestamp</t>
+  </si>
+  <si>
+    <t>Dashboard.addProductToCart</t>
+  </si>
+  <si>
     <t>iphone 13 pro</t>
   </si>
   <si>
-    <t>Sathish Reddy</t>
-  </si>
-  <si>
-    <t>India</t>
-  </si>
-  <si>
-    <t>ExpectedCartCount</t>
-  </si>
-  <si>
-    <t>CardNumber</t>
-  </si>
-  <si>
-    <t>Month</t>
-  </si>
-  <si>
-    <t>Date</t>
-  </si>
-  <si>
-    <t>Name</t>
-  </si>
-  <si>
-    <t>ExpectedQty</t>
-  </si>
-  <si>
-    <t>ZARA COAT 3</t>
-  </si>
-  <si>
-    <t>Sathish Reddy Sandhi</t>
-  </si>
-  <si>
-    <t>1234567898765432</t>
-  </si>
-  <si>
-    <t>09</t>
-  </si>
-  <si>
-    <t>E2ETest</t>
-  </si>
-  <si>
-    <t>CompletedFlow</t>
-  </si>
-  <si>
-    <t>Status</t>
-  </si>
-  <si>
-    <t>Cart.goToCheckout</t>
+    <t>Clothes</t>
+  </si>
+  <si>
+    <t>Execution</t>
+  </si>
+  <si>
+    <t>PASS</t>
+  </si>
+  <si>
+    <t>Dashboard.goToCartPage</t>
+  </si>
+  <si>
+    <t>Completed Execution</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="0"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="yyyy-MM-dd HH:mm:ss"/>
+  </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -113,13 +165,8 @@
       <patternFill patternType="gray125"/>
     </fill>
     <fill>
-      <patternFill patternType="none">
-        <fgColor indexed="17"/>
-      </patternFill>
-    </fill>
-    <fill>
       <patternFill patternType="solid">
-        <fgColor indexed="17"/>
+        <fgColor indexed="10"/>
       </patternFill>
     </fill>
     <fill>
@@ -128,8 +175,13 @@
       </patternFill>
     </fill>
     <fill>
+      <patternFill patternType="none">
+        <fgColor indexed="17"/>
+      </patternFill>
+    </fill>
+    <fill>
       <patternFill patternType="solid">
-        <fgColor indexed="10"/>
+        <fgColor indexed="17"/>
       </patternFill>
     </fill>
   </fills>
@@ -145,14 +197,65 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="58">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="true"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="true"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="true"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="true"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="true"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="true"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="true"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="true"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="true"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="true"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="true"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="true"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="true"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="true"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="true"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="true"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="true"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="true"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="true"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="true"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="true"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="true"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="true"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="true"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="true"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="true"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="true"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -432,11 +535,80 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CF2D4A01-FD8A-4C00-8AEF-6100DA0E02DE}">
-  <dimension ref="A1:B3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D4687A51-E3F6-4959-AD9A-99F0B4444C26}">
+  <dimension ref="A1:D4"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="14.1796875"/>
+    <col min="2" max="2" customWidth="true" width="29.90625"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="0">
+        <v>25</v>
+      </c>
+      <c r="B1" t="s" s="0">
+        <v>26</v>
+      </c>
+      <c r="C1" t="s" s="0">
+        <v>27</v>
+      </c>
+      <c r="D1" t="s" s="0">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="B2" t="s" s="0">
+        <v>35</v>
+      </c>
+      <c r="C2" t="s" s="52">
+        <v>33</v>
+      </c>
+      <c r="D2" s="53" t="n">
+        <v>46107.07114574074</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="B3" t="s" s="0">
+        <v>35</v>
+      </c>
+      <c r="C3" t="s" s="54">
+        <v>33</v>
+      </c>
+      <c r="D3" s="55" t="n">
+        <v>46107.07139671296</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="B4" t="s" s="0">
+        <v>35</v>
+      </c>
+      <c r="C4" t="s" s="56">
+        <v>33</v>
+      </c>
+      <c r="D4" s="57" t="n">
+        <v>46107.071665972224</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CF2D4A01-FD8A-4C00-8AEF-6100DA0E02DE}">
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" customWidth="true" width="37.54296875"/>
     <col min="2" max="2" customWidth="true" width="23.08984375"/>
   </cols>
   <sheetData>
@@ -445,33 +617,42 @@
         <v>0</v>
       </c>
       <c r="B1" t="s" s="0">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="B2" s="1">
+        <v>30</v>
+      </c>
+      <c r="B2" s="0">
         <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="s" s="0">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="B3" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A4" t="s" s="0">
+        <v>31</v>
+      </c>
+      <c r="B4" s="0">
         <v>1</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{334CF848-C880-4642-954D-864DF5E51C2D}">
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" customWidth="true" width="19.90625"/>
@@ -482,22 +663,30 @@
         <v>0</v>
       </c>
       <c r="B1" t="s" s="0">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="B2" s="1">
+        <v>30</v>
+      </c>
+      <c r="B2" s="0">
         <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="s" s="0">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="B3" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A4" t="s" s="0">
+        <v>31</v>
+      </c>
+      <c r="B4" s="0">
         <v>1</v>
       </c>
     </row>
@@ -507,9 +696,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B2AF52E-5086-43AC-9E41-3304A02A9C8C}">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" customWidth="true" width="23.81640625"/>
@@ -520,19 +709,19 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="B1" t="s" s="0">
         <v>7</v>
       </c>
-      <c r="B1" t="s" s="0">
+      <c r="C1" t="s" s="0">
         <v>8</v>
       </c>
-      <c r="C1" t="s" s="0">
+      <c r="D1" t="s" s="0">
+        <v>1</v>
+      </c>
+      <c r="E1" t="s" s="0">
         <v>9</v>
-      </c>
-      <c r="D1" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="E1" t="s" s="0">
-        <v>10</v>
       </c>
       <c r="F1" t="s" s="0">
         <v>2</v>
@@ -540,7 +729,7 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B2" s="1">
         <v>12</v>
@@ -552,18 +741,18 @@
         <v>274</v>
       </c>
       <c r="E2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F2" t="s" s="0">
         <v>4</v>
-      </c>
-      <c r="F2" t="s" s="0">
-        <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C3" s="1">
         <v>10</v>
@@ -572,10 +761,30 @@
         <v>294</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F3" t="s" s="0">
-        <v>5</v>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A4" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C4" s="1">
+        <v>15</v>
+      </c>
+      <c r="D4" s="1">
+        <v>934</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="F4" t="s" s="0">
+        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -583,9 +792,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4E14915E-E896-4209-8E48-035EA63E22E1}">
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" customWidth="true" width="16.1796875"/>
@@ -597,22 +806,30 @@
         <v>0</v>
       </c>
       <c r="B1" t="s" s="0">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="B2" s="1">
+        <v>30</v>
+      </c>
+      <c r="B2" s="0">
         <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="s" s="0">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="B3" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A4" t="s" s="0">
+        <v>31</v>
+      </c>
+      <c r="B4" s="0">
         <v>1</v>
       </c>
     </row>
@@ -622,52 +839,44 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F7FAC67C-2142-481E-8C57-BF49024F7BB1}">
-  <dimension ref="A1:C5"/>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EF8EAE46-4B76-4386-9505-380624A1252D}">
+  <dimension ref="A1:B4"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="2" max="2" customWidth="true" width="22.54296875"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="s" s="2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A1" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="B1" t="s" s="0">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A2" t="s" s="0">
         <v>16</v>
       </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="s" s="3">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="3">
+      <c r="B2" t="s" s="0">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="s" s="0">
         <v>16</v>
       </c>
       <c r="B3" t="s" s="0">
         <v>17</v>
       </c>
-      <c r="C3" t="s" s="4">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="4">
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" t="s" s="0">
         <v>16</v>
       </c>
       <c r="B4" t="s" s="0">
         <v>17</v>
-      </c>
-      <c r="C4" t="s" s="5">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="s" s="0">
-        <v>16</v>
-      </c>
-      <c r="B5" t="s" s="0">
-        <v>19</v>
-      </c>
-      <c r="C5" t="s" s="6">
-        <v>18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>